<commit_message>
docs: disponibiliza modelo limpo com formatação original preservada
</commit_message>
<xml_diff>
--- a/public/main.xlsx
+++ b/public/main.xlsx
@@ -3,8 +3,11 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Modelo" sheetId="1" r:id="rId1"/>
+    <sheet name="Digitalizado PDF" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Digitalizado PDF'!A2:M2</definedName>
+  </definedNames>
 </workbook>
 </file>
 
@@ -32,10 +35,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="3">
+  <numFmts count="1">
     <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-    <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
-    <numFmt numFmtId="165" formatCode="hh:mm"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -401,125 +402,54 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:AF2"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>RASTREADOR</v>
-      </c>
-      <c r="B1" t="str">
-        <v>DADOS MATRIZ PDR</v>
-      </c>
-      <c r="C1" t="str">
-        <v>DADOS FILIAL PDR</v>
-      </c>
-      <c r="D1" t="str">
-        <v>REGISTRO DE CARGAS</v>
-      </c>
-    </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>CÓDIGO VISITA</v>
+        <v>RAZÃO SOCIAL FILIAL PDR</v>
       </c>
       <c r="B2" t="str">
-        <v>REGIONAL MATRIZ</v>
+        <v>CNPJ FILIAL PDR</v>
       </c>
       <c r="C2" t="str">
-        <v>REGIONAL FILIAL</v>
+        <v>DATA</v>
       </c>
       <c r="D2" t="str">
-        <v>ID</v>
+        <v>HORÁRIO</v>
       </c>
       <c r="E2" t="str">
-        <v>EMPRESA HARVEST</v>
+        <v>TIPO DOCUMENTO</v>
       </c>
       <c r="F2" t="str">
-        <v>OPERAÇÃO</v>
+        <v>NÚMERO DOCUMENTO</v>
       </c>
       <c r="G2" t="str">
-        <v>DISTRITO MATRIZ</v>
+        <v>PESO LÍQUIDO (KG)</v>
       </c>
       <c r="H2" t="str">
-        <v>RAZÃO SOCIAL MATRIZ PDR</v>
+        <v>PESO LÍQUIDO C/ DESCONTO (KG)</v>
       </c>
       <c r="I2" t="str">
-        <v>CNPJ MATRIZ PDR</v>
+        <v>RESULTADO DO TESTE ACOMPANHADO</v>
       </c>
       <c r="J2" t="str">
-        <v>DISTRITO FILIAL</v>
+        <v>PRODUTOR</v>
       </c>
       <c r="K2" t="str">
-        <v>UF FILIAL</v>
+        <v>CNPJ/CPF PRODUTOR</v>
       </c>
       <c r="L2" t="str">
-        <v>CIDADE FILIAL</v>
+        <v>PLACA DO CAMINHÃO</v>
       </c>
       <c r="M2" t="str">
-        <v>RAZÃO SOCIAL FILIAL PDR</v>
-      </c>
-      <c r="N2" t="str">
-        <v>CNPJ FILIAL PDR</v>
-      </c>
-      <c r="O2" t="str">
-        <v>DATA</v>
-      </c>
-      <c r="P2" t="str">
-        <v>HORÁRIO</v>
-      </c>
-      <c r="Q2" t="str">
-        <v>TIPO DOCUMENTO</v>
-      </c>
-      <c r="R2" t="str">
-        <v>NÚMERO DOCUMENTO</v>
-      </c>
-      <c r="S2" t="str">
-        <v>PESO LÍQUIDO (KG)</v>
-      </c>
-      <c r="T2" t="str">
-        <v>PESO LÍQUIDO C/ DESCONTO (KG)</v>
-      </c>
-      <c r="U2" t="str">
-        <v>RESULTADO DO TESTE ACOMPANHADO</v>
-      </c>
-      <c r="V2" t="str">
-        <v>PRODUTOR</v>
-      </c>
-      <c r="W2" t="str">
-        <v>CNPJ/CPF PRODUTOR</v>
-      </c>
-      <c r="X2" t="str">
-        <v>PLACA DO CAMINHÃO</v>
-      </c>
-      <c r="Y2" t="str">
         <v>NÃO ACOMPANHADA</v>
-      </c>
-      <c r="Z2" t="str">
-        <v>HORARIO SISTÊMICO</v>
-      </c>
-      <c r="AA2" t="str">
-        <v>TIPO DA VISITA</v>
-      </c>
-      <c r="AB2" t="str">
-        <v>OBSERVAÇÃO</v>
-      </c>
-      <c r="AC2" t="str">
-        <v>DATA CADASTRO</v>
-      </c>
-      <c r="AD2" t="str">
-        <v>LATITUDE</v>
-      </c>
-      <c r="AE2" t="str">
-        <v>LONGITUDE</v>
-      </c>
-      <c r="AF2" t="str">
-        <v>rateio</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="N1:AF1"/>
-    <mergeCell ref="H1:M1"/>
-    <mergeCell ref="D1:G1"/>
+  <autoFilter ref="A2:M2"/>
+  <mergeCells count="2">
+    <mergeCell ref="C1:M1"/>
+    <mergeCell ref="A1:B1"/>
   </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:AF2"/>
   </ignoredErrors>

</xml_diff>